<commit_message>
removed duplicate/raw reward comparison outputs
</commit_message>
<xml_diff>
--- a/proposed/results/training_tables/emergency_training_results.xlsx
+++ b/proposed/results/training_tables/emergency_training_results.xlsx
@@ -448,10 +448,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>7604.2089</v>
+        <v>6615.2856</v>
       </c>
       <c r="C2" t="n">
-        <v>152.0842</v>
+        <v>132.3057</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -459,7 +459,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.5888</v>
+        <v>0.5962</v>
       </c>
     </row>
     <row r="3">
@@ -467,10 +467,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>9314.459999999999</v>
+        <v>6340.5348</v>
       </c>
       <c r="C3" t="n">
-        <v>186.2892</v>
+        <v>126.8107</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.0566</v>
+        <v>0.0502</v>
       </c>
     </row>
     <row r="4">
@@ -486,10 +486,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>8973.387500000001</v>
+        <v>4921.7329</v>
       </c>
       <c r="C4" t="n">
-        <v>179.4678</v>
+        <v>98.43470000000001</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.0476</v>
+        <v>0.0496</v>
       </c>
     </row>
     <row r="5">
@@ -505,10 +505,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>9095.492200000001</v>
+        <v>6562.0543</v>
       </c>
       <c r="C5" t="n">
-        <v>181.9098</v>
+        <v>131.2411</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.0513</v>
+        <v>0.0559</v>
       </c>
     </row>
     <row r="6">
@@ -524,10 +524,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>10422.2809</v>
+        <v>6928.039</v>
       </c>
       <c r="C6" t="n">
-        <v>208.4456</v>
+        <v>138.5608</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.1576</v>
+        <v>0.1609</v>
       </c>
     </row>
     <row r="7">
@@ -543,10 +543,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>7771.2526</v>
+        <v>3492.4983</v>
       </c>
       <c r="C7" t="n">
-        <v>155.4251</v>
+        <v>69.84999999999999</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.0593</v>
+        <v>0.0526</v>
       </c>
     </row>
     <row r="8">
@@ -562,10 +562,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>9961.9931</v>
+        <v>6813.8505</v>
       </c>
       <c r="C8" t="n">
-        <v>199.2399</v>
+        <v>136.277</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.0525</v>
+        <v>0.0569</v>
       </c>
     </row>
     <row r="9">
@@ -581,10 +581,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>8049.9372</v>
+        <v>4144.0716</v>
       </c>
       <c r="C9" t="n">
-        <v>160.9987</v>
+        <v>82.8814</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.0596</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="10">
@@ -600,10 +600,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>8829.4828</v>
+        <v>4706.6534</v>
       </c>
       <c r="C10" t="n">
-        <v>176.5897</v>
+        <v>94.1331</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.1471</v>
+        <v>0.1622</v>
       </c>
     </row>
     <row r="11">
@@ -619,10 +619,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>7597.4596</v>
+        <v>3580.494</v>
       </c>
       <c r="C11" t="n">
-        <v>151.9492</v>
+        <v>71.6099</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.0498</v>
+        <v>0.0514</v>
       </c>
     </row>
     <row r="12">
@@ -638,10 +638,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>7434.9988</v>
+        <v>4358.8457</v>
       </c>
       <c r="C12" t="n">
-        <v>148.7</v>
+        <v>87.1769</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.0625</v>
+        <v>0.0584</v>
       </c>
     </row>
     <row r="13">
@@ -657,10 +657,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>8829.573399999999</v>
+        <v>5654.3342</v>
       </c>
       <c r="C13" t="n">
-        <v>176.5915</v>
+        <v>113.0867</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.0571</v>
+        <v>0.0609</v>
       </c>
     </row>
     <row r="14">
@@ -676,10 +676,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>8541.5738</v>
+        <v>4239.0056</v>
       </c>
       <c r="C14" t="n">
-        <v>170.8315</v>
+        <v>84.7801</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.165</v>
+        <v>0.1447</v>
       </c>
     </row>
     <row r="15">
@@ -695,10 +695,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>10231.9779</v>
+        <v>7231.2794</v>
       </c>
       <c r="C15" t="n">
-        <v>204.6396</v>
+        <v>144.6256</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.0553</v>
+        <v>0.0492</v>
       </c>
     </row>
     <row r="16">
@@ -714,10 +714,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>8308.5697</v>
+        <v>4729.2811</v>
       </c>
       <c r="C16" t="n">
-        <v>166.1714</v>
+        <v>94.5856</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.0513</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="17">
@@ -733,10 +733,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>8091.6182</v>
+        <v>4388.6954</v>
       </c>
       <c r="C17" t="n">
-        <v>161.8324</v>
+        <v>87.7739</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.056</v>
+        <v>0.0519</v>
       </c>
     </row>
     <row r="18">
@@ -752,10 +752,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>11372.6405</v>
+        <v>8872.332200000001</v>
       </c>
       <c r="C18" t="n">
-        <v>227.4528</v>
+        <v>177.4466</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.152</v>
+        <v>0.1633</v>
       </c>
     </row>
     <row r="19">
@@ -771,10 +771,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>7372.8437</v>
+        <v>3853.6569</v>
       </c>
       <c r="C19" t="n">
-        <v>147.4569</v>
+        <v>77.0731</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.0513</v>
+        <v>0.0786</v>
       </c>
     </row>
     <row r="20">
@@ -790,10 +790,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>7840.7257</v>
+        <v>3987.3513</v>
       </c>
       <c r="C20" t="n">
-        <v>156.8145</v>
+        <v>79.747</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.1349</v>
+        <v>0.0577</v>
       </c>
     </row>
     <row r="21">
@@ -809,10 +809,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>10078.4253</v>
+        <v>7027.1647</v>
       </c>
       <c r="C21" t="n">
-        <v>201.5685</v>
+        <v>140.5433</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -820,7 +820,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.0799</v>
+        <v>0.067</v>
       </c>
     </row>
     <row r="22">
@@ -828,10 +828,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>11124.0703</v>
+        <v>6799.1594</v>
       </c>
       <c r="C22" t="n">
-        <v>222.4814</v>
+        <v>135.9832</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.1612</v>
+        <v>0.1964</v>
       </c>
     </row>
     <row r="23">
@@ -847,10 +847,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>10706.3444</v>
+        <v>8206.2729</v>
       </c>
       <c r="C23" t="n">
-        <v>214.1269</v>
+        <v>164.1255</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.0573</v>
+        <v>0.0703</v>
       </c>
     </row>
     <row r="24">
@@ -866,10 +866,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>10312.7183</v>
+        <v>7301.7094</v>
       </c>
       <c r="C24" t="n">
-        <v>206.2544</v>
+        <v>146.0342</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.0554</v>
+        <v>0.0701</v>
       </c>
     </row>
     <row r="25">
@@ -885,10 +885,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>12993.3775</v>
+        <v>10478.4406</v>
       </c>
       <c r="C25" t="n">
-        <v>259.8675</v>
+        <v>209.5688</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.0549</v>
+        <v>0.0728</v>
       </c>
     </row>
     <row r="26">
@@ -904,10 +904,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>10799.3115</v>
+        <v>8148.2075</v>
       </c>
       <c r="C26" t="n">
-        <v>215.9862</v>
+        <v>162.9641</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.1543</v>
+        <v>0.1966</v>
       </c>
     </row>
     <row r="27">
@@ -923,10 +923,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>10580.5369</v>
+        <v>4820.9969</v>
       </c>
       <c r="C27" t="n">
-        <v>211.6107</v>
+        <v>96.4199</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -934,7 +934,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.0512</v>
+        <v>0.0704</v>
       </c>
     </row>
     <row r="28">
@@ -942,10 +942,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>9599.1013</v>
+        <v>6797.8297</v>
       </c>
       <c r="C28" t="n">
-        <v>191.982</v>
+        <v>135.9566</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.0523</v>
+        <v>0.07149999999999999</v>
       </c>
     </row>
     <row r="29">
@@ -961,10 +961,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>7094.2688</v>
+        <v>2690.4032</v>
       </c>
       <c r="C29" t="n">
-        <v>141.8854</v>
+        <v>53.8081</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.0495</v>
+        <v>0.0692</v>
       </c>
     </row>
     <row r="30">
@@ -980,10 +980,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>7738.4324</v>
+        <v>3462.633</v>
       </c>
       <c r="C30" t="n">
-        <v>154.7686</v>
+        <v>69.2527</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -991,7 +991,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.1548</v>
+        <v>0.1969</v>
       </c>
     </row>
     <row r="31">
@@ -999,10 +999,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>13419.1683</v>
+        <v>11197.6864</v>
       </c>
       <c r="C31" t="n">
-        <v>268.3834</v>
+        <v>223.9537</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.0557</v>
+        <v>0.0727</v>
       </c>
     </row>
     <row r="32">
@@ -1018,10 +1018,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>12043.1525</v>
+        <v>8109.1505</v>
       </c>
       <c r="C32" t="n">
-        <v>240.8631</v>
+        <v>162.183</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.0611</v>
+        <v>0.0694</v>
       </c>
     </row>
     <row r="33">
@@ -1037,10 +1037,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>12873.9019</v>
+        <v>10382.6019</v>
       </c>
       <c r="C33" t="n">
-        <v>257.478</v>
+        <v>207.652</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.066</v>
+        <v>0.0726</v>
       </c>
     </row>
     <row r="34">
@@ -1056,10 +1056,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>9295.931200000001</v>
+        <v>6562.4082</v>
       </c>
       <c r="C34" t="n">
-        <v>185.9186</v>
+        <v>131.2482</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.1603</v>
+        <v>0.1987</v>
       </c>
     </row>
     <row r="35">
@@ -1075,10 +1075,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="n">
-        <v>8918.400799999999</v>
+        <v>5966.5415</v>
       </c>
       <c r="C35" t="n">
-        <v>178.368</v>
+        <v>119.3308</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.0636</v>
+        <v>0.07049999999999999</v>
       </c>
     </row>
     <row r="36">
@@ -1094,10 +1094,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="n">
-        <v>11665.0149</v>
+        <v>9071.6729</v>
       </c>
       <c r="C36" t="n">
-        <v>233.3003</v>
+        <v>181.4335</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.0511</v>
+        <v>0.0712</v>
       </c>
     </row>
     <row r="37">
@@ -1113,10 +1113,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="n">
-        <v>6993.9354</v>
+        <v>2179.8597</v>
       </c>
       <c r="C37" t="n">
-        <v>139.8787</v>
+        <v>43.5972</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.0487</v>
+        <v>0.0658</v>
       </c>
     </row>
     <row r="38">
@@ -1132,10 +1132,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>13313.4206</v>
+        <v>9039.111199999999</v>
       </c>
       <c r="C38" t="n">
-        <v>266.2684</v>
+        <v>180.7822</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.1479</v>
+        <v>0.1972</v>
       </c>
     </row>
     <row r="39">
@@ -1151,10 +1151,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="n">
-        <v>9996.0172</v>
+        <v>5591.1492</v>
       </c>
       <c r="C39" t="n">
-        <v>199.9203</v>
+        <v>111.823</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.0524</v>
+        <v>0.0678</v>
       </c>
     </row>
     <row r="40">
@@ -1170,10 +1170,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>11399.9496</v>
+        <v>5343.1695</v>
       </c>
       <c r="C40" t="n">
-        <v>227.999</v>
+        <v>106.8634</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.0513</v>
+        <v>0.06710000000000001</v>
       </c>
     </row>
     <row r="41">
@@ -1189,10 +1189,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>10453.4242</v>
+        <v>7582.6726</v>
       </c>
       <c r="C41" t="n">
-        <v>209.0685</v>
+        <v>151.6535</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.051</v>
+        <v>0.07340000000000001</v>
       </c>
     </row>
     <row r="42">
@@ -1208,10 +1208,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>9071.960800000001</v>
+        <v>6218.84</v>
       </c>
       <c r="C42" t="n">
-        <v>181.4392</v>
+        <v>124.3768</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.1566</v>
+        <v>0.194</v>
       </c>
     </row>
     <row r="43">
@@ -1227,10 +1227,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>9899.924199999999</v>
+        <v>6886.8741</v>
       </c>
       <c r="C43" t="n">
-        <v>197.9985</v>
+        <v>137.7375</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.0641</v>
+        <v>0.0709</v>
       </c>
     </row>
     <row r="44">
@@ -1246,10 +1246,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="n">
-        <v>7529.8612</v>
+        <v>3329.3306</v>
       </c>
       <c r="C44" t="n">
-        <v>150.5972</v>
+        <v>66.5866</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.0516</v>
+        <v>0.0688</v>
       </c>
     </row>
     <row r="45">
@@ -1265,10 +1265,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>9961.164500000001</v>
+        <v>6096.7103</v>
       </c>
       <c r="C45" t="n">
-        <v>199.2233</v>
+        <v>121.9342</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.0612</v>
+        <v>0.0738</v>
       </c>
     </row>
     <row r="46">
@@ -1284,10 +1284,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>8401.374599999999</v>
+        <v>4471.3039</v>
       </c>
       <c r="C46" t="n">
-        <v>168.0275</v>
+        <v>89.42610000000001</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.1541</v>
+        <v>0.1971</v>
       </c>
     </row>
     <row r="47">
@@ -1303,10 +1303,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="n">
-        <v>9636.747499999999</v>
+        <v>6922.2533</v>
       </c>
       <c r="C47" t="n">
-        <v>192.7349</v>
+        <v>138.4451</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.0551</v>
+        <v>0.0725</v>
       </c>
     </row>
     <row r="48">
@@ -1322,10 +1322,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="n">
-        <v>9906.184800000001</v>
+        <v>6845.2401</v>
       </c>
       <c r="C48" t="n">
-        <v>198.1237</v>
+        <v>136.9048</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.0555</v>
+        <v>0.07240000000000001</v>
       </c>
     </row>
     <row r="49">
@@ -1341,10 +1341,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="n">
-        <v>10176.282</v>
+        <v>7267.2354</v>
       </c>
       <c r="C49" t="n">
-        <v>203.5256</v>
+        <v>145.3447</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.0578</v>
+        <v>0.07190000000000001</v>
       </c>
     </row>
     <row r="50">
@@ -1360,10 +1360,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="n">
-        <v>12563.0449</v>
+        <v>10063.0449</v>
       </c>
       <c r="C50" t="n">
-        <v>251.2609</v>
+        <v>201.2609</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.1574</v>
+        <v>0.1743</v>
       </c>
     </row>
     <row r="51">
@@ -1379,10 +1379,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="n">
-        <v>7986.4612</v>
+        <v>4742.4043</v>
       </c>
       <c r="C51" t="n">
-        <v>159.7292</v>
+        <v>94.8481</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.0547</v>
+        <v>0.0542</v>
       </c>
     </row>
     <row r="52">
@@ -1398,10 +1398,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="n">
-        <v>8175.8951</v>
+        <v>4469.0507</v>
       </c>
       <c r="C52" t="n">
-        <v>163.5179</v>
+        <v>89.381</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1409,7 +1409,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.0516</v>
+        <v>0.053</v>
       </c>
     </row>
     <row r="53">
@@ -1417,10 +1417,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="n">
-        <v>10258.0306</v>
+        <v>6518.7148</v>
       </c>
       <c r="C53" t="n">
-        <v>205.1606</v>
+        <v>130.3743</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1428,7 +1428,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0.0533</v>
+        <v>0.054</v>
       </c>
     </row>
     <row r="54">
@@ -1436,10 +1436,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="n">
-        <v>8323.9509</v>
+        <v>5568.5633</v>
       </c>
       <c r="C54" t="n">
-        <v>166.479</v>
+        <v>111.3713</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0.1584</v>
+        <v>0.1664</v>
       </c>
     </row>
     <row r="55">
@@ -1455,10 +1455,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="n">
-        <v>11385.2375</v>
+        <v>7231.4112</v>
       </c>
       <c r="C55" t="n">
-        <v>227.7047</v>
+        <v>144.6282</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.0533</v>
+        <v>0.054</v>
       </c>
     </row>
     <row r="56">
@@ -1474,10 +1474,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="n">
-        <v>7167.9092</v>
+        <v>2561.7299</v>
       </c>
       <c r="C56" t="n">
-        <v>143.3582</v>
+        <v>51.2346</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.0517</v>
+        <v>0.0471</v>
       </c>
     </row>
     <row r="57">
@@ -1493,10 +1493,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="n">
-        <v>12239.6378</v>
+        <v>9653.9323</v>
       </c>
       <c r="C57" t="n">
-        <v>244.7928</v>
+        <v>193.0786</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>0.0625</v>
+        <v>0.0725</v>
       </c>
     </row>
     <row r="58">
@@ -1512,10 +1512,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="n">
-        <v>9734.145699999999</v>
+        <v>6234.5275</v>
       </c>
       <c r="C58" t="n">
-        <v>194.6829</v>
+        <v>124.6905</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.1534</v>
+        <v>0.1491</v>
       </c>
     </row>
     <row r="59">
@@ -1531,10 +1531,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="n">
-        <v>7545.5889</v>
+        <v>3089.1582</v>
       </c>
       <c r="C59" t="n">
-        <v>150.9118</v>
+        <v>61.7832</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1542,7 +1542,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.0472</v>
+        <v>0.0483</v>
       </c>
     </row>
     <row r="60">
@@ -1550,10 +1550,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="n">
-        <v>8465.186600000001</v>
+        <v>4158.5684</v>
       </c>
       <c r="C60" t="n">
-        <v>169.3037</v>
+        <v>83.17140000000001</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.0477</v>
+        <v>0.0505</v>
       </c>
     </row>
     <row r="61">
@@ -1569,10 +1569,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="n">
-        <v>11964.411</v>
+        <v>8164.1935</v>
       </c>
       <c r="C61" t="n">
-        <v>239.2882</v>
+        <v>163.2839</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -1580,7 +1580,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.0511</v>
+        <v>0.0517</v>
       </c>
     </row>
     <row r="62">
@@ -1588,10 +1588,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="n">
-        <v>12523.1765</v>
+        <v>8794.8177</v>
       </c>
       <c r="C62" t="n">
-        <v>250.4635</v>
+        <v>175.8964</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.1565</v>
+        <v>0.153</v>
       </c>
     </row>
     <row r="63">
@@ -1607,10 +1607,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="n">
-        <v>11065.8113</v>
+        <v>7396.8521</v>
       </c>
       <c r="C63" t="n">
-        <v>221.3162</v>
+        <v>147.937</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.0531</v>
       </c>
     </row>
     <row r="64">
@@ -1626,10 +1626,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="n">
-        <v>10006.9135</v>
+        <v>7160.37</v>
       </c>
       <c r="C64" t="n">
-        <v>200.1383</v>
+        <v>143.2074</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.0631</v>
+        <v>0.0537</v>
       </c>
     </row>
     <row r="65">
@@ -1645,10 +1645,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="n">
-        <v>7432.259</v>
+        <v>3214.0992</v>
       </c>
       <c r="C65" t="n">
-        <v>148.6452</v>
+        <v>64.282</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -1656,7 +1656,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0.0598</v>
+        <v>0.0473</v>
       </c>
     </row>
     <row r="66">
@@ -1664,10 +1664,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="n">
-        <v>10433.4191</v>
+        <v>3773.8954</v>
       </c>
       <c r="C66" t="n">
-        <v>208.6684</v>
+        <v>75.47790000000001</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>0.1592</v>
+        <v>0.1526</v>
       </c>
     </row>
     <row r="67">
@@ -1683,10 +1683,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="n">
-        <v>8546.082399999999</v>
+        <v>4886.6505</v>
       </c>
       <c r="C67" t="n">
-        <v>170.9216</v>
+        <v>97.733</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1694,7 +1694,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>0.0525</v>
+        <v>0.052</v>
       </c>
     </row>
     <row r="68">
@@ -1702,10 +1702,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="n">
-        <v>7525.9086</v>
+        <v>3432.9892</v>
       </c>
       <c r="C68" t="n">
-        <v>150.5182</v>
+        <v>68.6598</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>0.0474</v>
+        <v>0.0509</v>
       </c>
     </row>
     <row r="69">
@@ -1721,10 +1721,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="n">
-        <v>10080.1049</v>
+        <v>6875.3221</v>
       </c>
       <c r="C69" t="n">
-        <v>201.6021</v>
+        <v>137.5064</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -1732,7 +1732,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>0.0499</v>
+        <v>0.0525</v>
       </c>
     </row>
     <row r="70">
@@ -1740,10 +1740,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="n">
-        <v>10860.6777</v>
+        <v>8136.0611</v>
       </c>
       <c r="C70" t="n">
-        <v>217.2136</v>
+        <v>162.7212</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0.1486</v>
+        <v>0.2093</v>
       </c>
     </row>
     <row r="71">
@@ -1759,10 +1759,10 @@
         <v>70</v>
       </c>
       <c r="B71" t="n">
-        <v>9139.8995</v>
+        <v>6379.3209</v>
       </c>
       <c r="C71" t="n">
-        <v>182.798</v>
+        <v>127.5864</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -1770,7 +1770,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0.0523</v>
+        <v>0.07679999999999999</v>
       </c>
     </row>
     <row r="72">
@@ -1778,10 +1778,10 @@
         <v>71</v>
       </c>
       <c r="B72" t="n">
-        <v>11803.0571</v>
+        <v>7653.6796</v>
       </c>
       <c r="C72" t="n">
-        <v>236.0611</v>
+        <v>153.0736</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>0.0521</v>
+        <v>0.0723</v>
       </c>
     </row>
     <row r="73">
@@ -1797,10 +1797,10 @@
         <v>72</v>
       </c>
       <c r="B73" t="n">
-        <v>7721.1751</v>
+        <v>3113.4245</v>
       </c>
       <c r="C73" t="n">
-        <v>154.4235</v>
+        <v>62.2685</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>0.0616</v>
+        <v>0.06909999999999999</v>
       </c>
     </row>
     <row r="74">
@@ -1816,10 +1816,10 @@
         <v>73</v>
       </c>
       <c r="B74" t="n">
-        <v>8525.7354</v>
+        <v>4868.2789</v>
       </c>
       <c r="C74" t="n">
-        <v>170.5147</v>
+        <v>97.3656</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.162</v>
+        <v>0.1908</v>
       </c>
     </row>
     <row r="75">
@@ -1835,10 +1835,10 @@
         <v>74</v>
       </c>
       <c r="B75" t="n">
-        <v>8336.2073</v>
+        <v>3810.293</v>
       </c>
       <c r="C75" t="n">
-        <v>166.7241</v>
+        <v>76.2059</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0.0603</v>
+        <v>0.056</v>
       </c>
     </row>
     <row r="76">
@@ -1854,10 +1854,10 @@
         <v>75</v>
       </c>
       <c r="B76" t="n">
-        <v>10145.6428</v>
+        <v>7593.6674</v>
       </c>
       <c r="C76" t="n">
-        <v>202.9129</v>
+        <v>151.8733</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0.0505</v>
+        <v>0.0579</v>
       </c>
     </row>
     <row r="77">
@@ -1873,10 +1873,10 @@
         <v>76</v>
       </c>
       <c r="B77" t="n">
-        <v>11602.7733</v>
+        <v>8201.307199999999</v>
       </c>
       <c r="C77" t="n">
-        <v>232.0555</v>
+        <v>164.0261</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>0.0531</v>
+        <v>0.0633</v>
       </c>
     </row>
     <row r="78">
@@ -1892,10 +1892,10 @@
         <v>77</v>
       </c>
       <c r="B78" t="n">
-        <v>8012.6645</v>
+        <v>4284.366</v>
       </c>
       <c r="C78" t="n">
-        <v>160.2533</v>
+        <v>85.68729999999999</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>0.1551</v>
+        <v>0.2043</v>
       </c>
     </row>
     <row r="79">
@@ -1911,10 +1911,10 @@
         <v>78</v>
       </c>
       <c r="B79" t="n">
-        <v>10215.2588</v>
+        <v>5562.6258</v>
       </c>
       <c r="C79" t="n">
-        <v>204.3052</v>
+        <v>111.2525</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>0.0537</v>
+        <v>0.073</v>
       </c>
     </row>
     <row r="80">
@@ -1930,10 +1930,10 @@
         <v>79</v>
       </c>
       <c r="B80" t="n">
-        <v>8260.5357</v>
+        <v>4764.0154</v>
       </c>
       <c r="C80" t="n">
-        <v>165.2107</v>
+        <v>95.2803</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>0.0499</v>
+        <v>0.0717</v>
       </c>
     </row>
     <row r="81">
@@ -1949,10 +1949,10 @@
         <v>80</v>
       </c>
       <c r="B81" t="n">
-        <v>9623.3863</v>
+        <v>6814.5826</v>
       </c>
       <c r="C81" t="n">
-        <v>192.4677</v>
+        <v>136.2917</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>0.0609</v>
+        <v>0.0745</v>
       </c>
     </row>
     <row r="82">
@@ -1968,10 +1968,10 @@
         <v>81</v>
       </c>
       <c r="B82" t="n">
-        <v>11621.8005</v>
+        <v>8712.0805</v>
       </c>
       <c r="C82" t="n">
-        <v>232.436</v>
+        <v>174.2416</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>0.1719</v>
+        <v>0.2134</v>
       </c>
     </row>
     <row r="83">
@@ -1987,10 +1987,10 @@
         <v>82</v>
       </c>
       <c r="B83" t="n">
-        <v>7533.9156</v>
+        <v>4025.0738</v>
       </c>
       <c r="C83" t="n">
-        <v>150.6783</v>
+        <v>80.50149999999999</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>0.0619</v>
+        <v>0.1255</v>
       </c>
     </row>
     <row r="84">
@@ -2006,10 +2006,10 @@
         <v>83</v>
       </c>
       <c r="B84" t="n">
-        <v>8142.7387</v>
+        <v>4636.4378</v>
       </c>
       <c r="C84" t="n">
-        <v>162.8548</v>
+        <v>92.72880000000001</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>0.0562</v>
+        <v>0.074</v>
       </c>
     </row>
     <row r="85">
@@ -2025,10 +2025,10 @@
         <v>84</v>
       </c>
       <c r="B85" t="n">
-        <v>9149.652400000001</v>
+        <v>5669.3107</v>
       </c>
       <c r="C85" t="n">
-        <v>182.993</v>
+        <v>113.3862</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -2036,7 +2036,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>0.0532</v>
+        <v>0.07439999999999999</v>
       </c>
     </row>
     <row r="86">
@@ -2044,10 +2044,10 @@
         <v>85</v>
       </c>
       <c r="B86" t="n">
-        <v>8389.1986</v>
+        <v>5392.5392</v>
       </c>
       <c r="C86" t="n">
-        <v>167.784</v>
+        <v>107.8508</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -2055,7 +2055,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>0.1569</v>
+        <v>0.1595</v>
       </c>
     </row>
     <row r="87">
@@ -2063,10 +2063,10 @@
         <v>86</v>
       </c>
       <c r="B87" t="n">
-        <v>8788.1531</v>
+        <v>5049.9967</v>
       </c>
       <c r="C87" t="n">
-        <v>175.7631</v>
+        <v>100.9999</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>0.0562</v>
+        <v>0.0665</v>
       </c>
     </row>
     <row r="88">
@@ -2082,10 +2082,10 @@
         <v>87</v>
       </c>
       <c r="B88" t="n">
-        <v>8928.472299999999</v>
+        <v>5205.6121</v>
       </c>
       <c r="C88" t="n">
-        <v>178.5694</v>
+        <v>104.1122</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>0.0611</v>
+        <v>0.0737</v>
       </c>
     </row>
     <row r="89">
@@ -2101,10 +2101,10 @@
         <v>88</v>
       </c>
       <c r="B89" t="n">
-        <v>9386.4362</v>
+        <v>6000.5439</v>
       </c>
       <c r="C89" t="n">
-        <v>187.7287</v>
+        <v>120.0109</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -2112,7 +2112,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>0.0619</v>
+        <v>0.0737</v>
       </c>
     </row>
     <row r="90">
@@ -2120,10 +2120,10 @@
         <v>89</v>
       </c>
       <c r="B90" t="n">
-        <v>12887.1164</v>
+        <v>10667.5164</v>
       </c>
       <c r="C90" t="n">
-        <v>257.7423</v>
+        <v>213.3503</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>0.171</v>
+        <v>0.2095</v>
       </c>
     </row>
     <row r="91">
@@ -2139,10 +2139,10 @@
         <v>90</v>
       </c>
       <c r="B91" t="n">
-        <v>7096.7738</v>
+        <v>3594.5182</v>
       </c>
       <c r="C91" t="n">
-        <v>141.9355</v>
+        <v>71.8904</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>0.0511</v>
+        <v>0.0727</v>
       </c>
     </row>
     <row r="92">
@@ -2158,10 +2158,10 @@
         <v>91</v>
       </c>
       <c r="B92" t="n">
-        <v>13135.793</v>
+        <v>8332.492399999999</v>
       </c>
       <c r="C92" t="n">
-        <v>262.7159</v>
+        <v>166.6498</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>0.0543</v>
+        <v>0.0746</v>
       </c>
     </row>
     <row r="93">
@@ -2177,10 +2177,10 @@
         <v>92</v>
       </c>
       <c r="B93" t="n">
-        <v>12351.1609</v>
+        <v>9729.5962</v>
       </c>
       <c r="C93" t="n">
-        <v>247.0232</v>
+        <v>194.5919</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>0.0527</v>
+        <v>0.0723</v>
       </c>
     </row>
     <row r="94">
@@ -2196,10 +2196,10 @@
         <v>93</v>
       </c>
       <c r="B94" t="n">
-        <v>8028.0755</v>
+        <v>3912.9776</v>
       </c>
       <c r="C94" t="n">
-        <v>160.5615</v>
+        <v>78.25960000000001</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>0.1524</v>
+        <v>0.2096</v>
       </c>
     </row>
     <row r="95">
@@ -2215,10 +2215,10 @@
         <v>94</v>
       </c>
       <c r="B95" t="n">
-        <v>9404.408600000001</v>
+        <v>6653.4139</v>
       </c>
       <c r="C95" t="n">
-        <v>188.0882</v>
+        <v>133.0683</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>0.0508</v>
+        <v>0.0689</v>
       </c>
     </row>
     <row r="96">
@@ -2234,10 +2234,10 @@
         <v>95</v>
       </c>
       <c r="B96" t="n">
-        <v>8028.4862</v>
+        <v>4620.4617</v>
       </c>
       <c r="C96" t="n">
-        <v>160.5697</v>
+        <v>92.4092</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2245,7 +2245,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>0.0592</v>
+        <v>0.0574</v>
       </c>
     </row>
     <row r="97">
@@ -2253,10 +2253,10 @@
         <v>96</v>
       </c>
       <c r="B97" t="n">
-        <v>13843.932</v>
+        <v>12823.932</v>
       </c>
       <c r="C97" t="n">
-        <v>276.8786</v>
+        <v>256.4786</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>0.0622</v>
+        <v>0.0592</v>
       </c>
     </row>
     <row r="98">
@@ -2272,10 +2272,10 @@
         <v>97</v>
       </c>
       <c r="B98" t="n">
-        <v>8132.6432</v>
+        <v>3557.2438</v>
       </c>
       <c r="C98" t="n">
-        <v>162.6529</v>
+        <v>71.14490000000001</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>0.1748</v>
+        <v>0.1686</v>
       </c>
     </row>
     <row r="99">
@@ -2291,10 +2291,10 @@
         <v>98</v>
       </c>
       <c r="B99" t="n">
-        <v>10424.0156</v>
+        <v>4260.3716</v>
       </c>
       <c r="C99" t="n">
-        <v>208.4803</v>
+        <v>85.20740000000001</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2302,7 +2302,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>0.0602</v>
+        <v>0.0567</v>
       </c>
     </row>
     <row r="100">
@@ -2310,10 +2310,10 @@
         <v>99</v>
       </c>
       <c r="B100" t="n">
-        <v>10854.3429</v>
+        <v>8354.3429</v>
       </c>
       <c r="C100" t="n">
-        <v>217.0869</v>
+        <v>167.0869</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -2321,7 +2321,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>0.0585</v>
+        <v>0.0598</v>
       </c>
     </row>
     <row r="101">
@@ -2329,10 +2329,10 @@
         <v>100</v>
       </c>
       <c r="B101" t="n">
-        <v>11406.0975</v>
+        <v>5773.9387</v>
       </c>
       <c r="C101" t="n">
-        <v>228.122</v>
+        <v>115.4788</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>0.0598</v>
+        <v>0.059</v>
       </c>
     </row>
   </sheetData>

</xml_diff>